<commit_message>
before trying to fix texting in dialogue
</commit_message>
<xml_diff>
--- a/card disdoc.xlsx
+++ b/card disdoc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5a34dfa97c331738/Documents/ilja/Unity/ld60/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="109" documentId="8_{0C438EE4-F750-43B6-8F91-DB4328E051E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{671BC9A9-A417-4AB5-81A5-6BD6FFC24168}"/>
+  <xr:revisionPtr revIDLastSave="144" documentId="8_{0C438EE4-F750-43B6-8F91-DB4328E051E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10702871-4A83-4D80-B4FF-851413DDB58A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{B625C734-B299-4013-86DD-D50F51382B50}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{B625C734-B299-4013-86DD-D50F51382B50}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="122">
   <si>
     <t>Hand (pts)</t>
   </si>
@@ -597,6 +597,74 @@
   </si>
   <si>
     <t>1 1 1 1 grants additoinal 200 points</t>
+  </si>
+  <si>
+    <t>interactable:</t>
+  </si>
+  <si>
+    <t>vynil player:</t>
+  </si>
+  <si>
+    <t>Every time i listen to this song, i feel like I am rotting alive
+But this pain is so beautiful and pleasant
+Perfect song for my funerals</t>
+  </si>
+  <si>
+    <t>It is my favorite part
+Silence moment before storm
+It sounds very sad
+It hopeful at the same time
+I used to call this feeling: melancholy
+Until i found out it has different meaning</t>
+  </si>
+  <si>
+    <t>its the end</t>
+  </si>
+  <si>
+    <t>Listening to this part, i feel only hatred
+out of onwhere 
+I dont know why</t>
+  </si>
+  <si>
+    <t>Character</t>
+  </si>
+  <si>
+    <t>First</t>
+  </si>
+  <si>
+    <t>after mom</t>
+  </si>
+  <si>
+    <t>after friend</t>
+  </si>
+  <si>
+    <t>after gf</t>
+  </si>
+  <si>
+    <t>I love my mother more than anything else in this world
+What i have become
+if she lost her hope...
+if Even she...
+How i caould...
+if she does, I surely do not deserve to live anymore</t>
+  </si>
+  <si>
+    <t>Maybe i am doing wrong.
+I've already made up my mind in any case.
+What people usually do in such moments?
+If think i need to call and say goodbye to some people</t>
+  </si>
+  <si>
+    <t>what is he not care about me at all this whole time?
+He is the person who new about me more than anyone else
+if even he didnt care about me, there nobody who does
+And i can pass away peacefully</t>
+  </si>
+  <si>
+    <t>We were perfect
+It sounds silly, but I think it really was
+Everybody think, it really was...
+I am jsut a selffish bitch</t>
   </si>
 </sst>
 </file>
@@ -640,7 +708,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -668,6 +736,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1864,7 +1936,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10006A7A-F87C-4A54-AC2B-0B8DC3F5EB25}">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -2081,6 +2153,73 @@
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
+    </row>
+    <row r="18" spans="13:18" x14ac:dyDescent="0.25">
+      <c r="M18" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="13:18" x14ac:dyDescent="0.25">
+      <c r="O19" s="10">
+        <v>0</v>
+      </c>
+      <c r="P19" s="10">
+        <v>0.25</v>
+      </c>
+      <c r="Q19" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="R19" s="10">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="20" spans="13:18" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M20" t="s">
+        <v>108</v>
+      </c>
+      <c r="O20" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="P20" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q20" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="R20" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="13:18" x14ac:dyDescent="0.25">
+      <c r="N23" t="s">
+        <v>114</v>
+      </c>
+      <c r="O23" t="s">
+        <v>115</v>
+      </c>
+      <c r="P23" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="24" spans="13:18" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M24" t="s">
+        <v>113</v>
+      </c>
+      <c r="N24" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="O24" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="P24" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q24" s="11" t="s">
+        <v>121</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="17">

</xml_diff>